<commit_message>
feat(web): Categories tab in Products; fix price book saving and the always-open catalog search
Categories can be listed, added in bulk, renamed and deleted under Products.
Price books failed to save once the customer was set back to None because an
empty string was sent as the customer id; empty selections are now omitted and
missing names or customers show a message. The catalog list opens with the
search box and closes on blur or Escape.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/crm-dashboard/tests/fixtures/product-import-template.xlsx
+++ b/crm-dashboard/tests/fixtures/product-import-template.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
   <si>
     <t>Manufacturer</t>
   </si>
@@ -33,6 +33,9 @@
     <t>Currencies</t>
   </si>
   <si>
+    <t>All categories</t>
+  </si>
+  <si>
     <t>Al Kuhaimi Metal Industries</t>
   </si>
   <si>
@@ -246,7 +249,7 @@
     <t>If it is not in the list, type the name anyway. Excel warns; continue. The import screen lists new names and offers to add them (or ask an administrator).</t>
   </si>
   <si>
-    <t>Pick from the drop-down after choosing the manufacturer: it shows that manufacturer's categories. A new category can be typed the same way.</t>
+    <t>Pick from the drop-down. With a manufacturer chosen it lists that manufacturer's categories; with Manufacturer blank it lists all categories and the import uses the default manufacturer chosen there. A new category can be typed the same way.</t>
   </si>
   <si>
     <t>The company the price came from, e.g. Ingram Micro. Blank uses the default chosen during import.</t>
@@ -654,16 +657,16 @@
   <sheetData>
     <row r="1" ht="30" customHeight="true">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>0</v>
@@ -672,13 +675,13 @@
         <v>1</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2">
@@ -6202,7 +6205,7 @@
       <formula1>Lists!$D$2:$D$28</formula1>
     </dataValidation>
     <dataValidation allowBlank="true" error="This category is not listed for the chosen manufacturer. Choose Yes to keep it; the import screen will offer to add it." errorStyle="warning" errorTitle="New category?" showErrorMessage="true" sqref="F2:F501" type="list">
-      <formula1>OFFSET(Lists!$B$1,MATCH($E2,Lists!$A:$A,0)-1,0,MAX(1,COUNTIF(Lists!$A:$A,$E2)),1)</formula1>
+      <formula1>IF($E2="",Lists!$H$2:$H$24,OFFSET(Lists!$B$1,MATCH($E2,Lists!$A:$A,0)-1,0,MAX(1,COUNTIF(Lists!$A:$A,$E2)),1))</formula1>
     </dataValidation>
   </dataValidations>
 </worksheet>
@@ -6218,23 +6221,23 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5">
@@ -6242,15 +6245,15 @@
         <v>0</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7">
@@ -6258,87 +6261,87 @@
         <v>1</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -6368,456 +6371,531 @@
       <c r="F1" t="s">
         <v>4</v>
       </c>
+      <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
-        <v>5</v>
-      </c>
       <c r="F2" t="s">
-        <v>55</v>
+        <v>56</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F3" t="s">
-        <v>56</v>
+        <v>57</v>
+      </c>
+      <c r="H3" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F4" t="s">
-        <v>57</v>
+        <v>58</v>
+      </c>
+      <c r="H4" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F5" t="s">
-        <v>58</v>
+        <v>59</v>
+      </c>
+      <c r="H5" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
       <c r="D6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>59</v>
+        <v>60</v>
+      </c>
+      <c r="H6" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F7" t="s">
-        <v>60</v>
+        <v>61</v>
+      </c>
+      <c r="H7" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D8" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="H8" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D9" t="s">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="H9" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="H10" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" t="s">
+        <v>28</v>
+      </c>
+      <c r="H11" t="s">
         <v>17</v>
-      </c>
-      <c r="B11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D11" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D12" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="H12" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D13" t="s">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="H13" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D14" t="s">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="H14" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D15" t="s">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="H15" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D16" t="s">
-        <v>35</v>
+        <v>36</v>
+      </c>
+      <c r="H16" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D17" t="s">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="H17" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" t="s">
+        <v>39</v>
+      </c>
+      <c r="H18" t="s">
         <v>24</v>
-      </c>
-      <c r="B18" t="s">
-        <v>26</v>
-      </c>
-      <c r="D18" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" t="s">
+        <v>40</v>
+      </c>
+      <c r="H19" t="s">
         <v>27</v>
-      </c>
-      <c r="B19" t="s">
-        <v>7</v>
-      </c>
-      <c r="D19" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B20" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D20" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="H20" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D21" t="s">
-        <v>42</v>
+        <v>43</v>
+      </c>
+      <c r="H21" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B22" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D22" t="s">
-        <v>43</v>
+        <v>44</v>
+      </c>
+      <c r="H22" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B23" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D23" t="s">
-        <v>45</v>
+        <v>46</v>
+      </c>
+      <c r="H23" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B24" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D24" t="s">
+        <v>48</v>
+      </c>
+      <c r="H24" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B25" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D25" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B26" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D26" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B27" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D27" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B28" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D28" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B29" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B32" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B34" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B35" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B36" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B37" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B38" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B39" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B41" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B42" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B43" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B45" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>